<commit_message>
Verification evaluation: override audit (conversation-driven, offline) + workbook Summary/predictions/emergency scoring/allow_followup=false
</commit_message>
<xml_diff>
--- a/ml/results/verification.xlsx
+++ b/ml/results/verification.xlsx
@@ -17,14 +17,14 @@
     <sheet name="SecondOpinion" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$H$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$H$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Predictions'!$A$1:$L$495</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Confusion'!$A$1:$F$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Errors'!$A$1:$E$219</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'RedFlags'!$A$1:$G$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Features'!$A$1:$P$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Provenance'!$A$1:$G$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'SecondOpinion'!$A$1:$F$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'SecondOpinion'!$A$1:$F$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -888,7 +888,7 @@
         <v>53</v>
       </c>
       <c r="E13" t="n">
-        <v>0.1083</v>
+        <v>0.1098</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
@@ -1087,33 +1087,1015 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>human_holdout</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>human_holdout.csv</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr">
+      <c r="H20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>override_rate (final != raw ML argmax)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>full pipeline vs raw ML argmax</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>see per-dataset rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>override_rate</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>unseen_tests.csv</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>full pipeline vs raw ML argmax</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>14</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.1429</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>not leaky</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>override_rate</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>redflag_holdout.csv</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>full pipeline vs raw ML argmax</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>22</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.3182</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>not leaky</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>override_rate</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>official_triage (exact-text CV OOF raw)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>full pipeline vs raw ML argmax</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>169</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.1006</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>in-sample rows (leaky for accuracy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>override_rate</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ALL (3 sets)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>full pipeline vs raw ML argmax</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>205</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.1268</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>per-dataset honesty above</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>override_stage_count</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0_model_version</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Production model differs from CV fold model (not a pipeline stage)</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>8</v>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>override_stage_count</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2_red_flag_bypass</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Stage 2 red-flag emergency bypass (rules)</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>16</v>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>override_stage_count</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2_module_decision</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Module decision (injury module: head hit -&gt; emergency)</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>override_stage_count</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>6.6_injury_sanity</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Stage 6.6 injury sanity</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>override_outcome</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>override corrected a raw-model error</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>21</v>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>override_outcome</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>broke</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>override broke a correct raw decision</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>5</v>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>human_holdout</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>human_holdout.csv</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
         <is>
           <t>missing - skipped</t>
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>llm_provider</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>live self-test</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>config</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>llm_model</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>live self-test</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>deepseek-v4-pro</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>config</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>llm_fast_model</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>live self-test</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>deepseek-flash</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>config</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>emergency_scoring_(a)_immediate_112</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>official_train</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>36</v>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>leaky - do not quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>emergency_scoring_(b)_confirm_then_yes</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>official_train</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ML/semantic flags</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>22</v>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>leaky - do not quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>emergency_scoring_(c)_missed</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>official_train</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>12</v>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>leaky - do not quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>emergency_recall_(a+b)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>official_train</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>rules + confirm-yes</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>70</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.8286</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.7238</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.8991</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>leaky - do not quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>emergency_scoring_(a)_immediate_112</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>official_val</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>leaky - do not quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>emergency_scoring_(b)_confirm_then_yes</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>official_val</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ML/semantic flags</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>13</v>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>leaky - do not quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>emergency_scoring_(c)_missed</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>official_val</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>leaky - do not quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>emergency_recall_(a+b)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>official_val</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>rules + confirm-yes</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>13</v>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.7719</v>
+      </c>
+      <c r="G43" t="n">
+        <v>1</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>leaky - do not quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>emergency_scoring_(a)_immediate_112</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>redflag_holdout</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>2</v>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>not leaky</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>emergency_scoring_(b)_confirm_then_yes</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>redflag_holdout</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ML/semantic flags</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>14</v>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>not leaky</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>emergency_scoring_(c)_missed</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>redflag_holdout</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>19</v>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>not leaky</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>emergency_recall_(a+b)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>redflag_holdout</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>rules + confirm-yes</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>35</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.4571</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.3047</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.6181</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>not leaky</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>emergency_scoring_(a)_immediate_112</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>unseen_tests</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>5</v>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>not leaky</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>emergency_scoring_(b)_confirm_then_yes</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>unseen_tests</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ML/semantic flags</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>not leaky</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>emergency_scoring_(c)_missed</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>unseen_tests</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>not leaky</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>emergency_recall_(a+b)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>unseen_tests</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>rules + confirm-yes</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>6</v>
+      </c>
+      <c r="E51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.6097</v>
+      </c>
+      <c r="G51" t="n">
+        <v>1</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>not leaky</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>allow_followup_false_accuracy</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>redflag_holdout</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>full pipeline (no followup)</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>53</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.3774</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.2594</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0.5119</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>not leaky</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>allow_followup_false_emergency_recall</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>redflag_holdout</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>full pipeline (no followup)</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>35</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0.0571</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.0158</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0.1861</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>not leaky</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>allow_followup_false_accuracy</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>unseen_tests</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>full pipeline (no followup)</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>30</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.5212</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0.8334</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>not leaky</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>allow_followup_false_emergency_recall</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>unseen_tests</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>full pipeline (no followup)</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>6</v>
+      </c>
+      <c r="E55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.6097</v>
+      </c>
+      <c r="G55" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>not leaky</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H20"/>
+  <autoFilter ref="A1:H55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24366,7 +25348,7 @@
       </c>
       <c r="E447" s="2" t="inlineStr">
         <is>
-          <t>teleconsultation</t>
+          <t>home_nursing</t>
         </is>
       </c>
       <c r="F447" s="2" t="n">
@@ -27044,13 +28026,13 @@
         <v>13</v>
       </c>
       <c r="C6" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F6" t="n">
         <v>44</v>
@@ -27166,13 +28148,13 @@
         <v>0.105</v>
       </c>
       <c r="C13" t="n">
-        <v>0.234</v>
+        <v>0.242</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>0.306</v>
+        <v>0.298</v>
       </c>
       <c r="F13" t="n">
         <v>0.355</v>
@@ -29378,7 +30360,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>teleconsultation</t>
+          <t>home_nursing</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -34154,7 +35136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -34208,7 +35190,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>value=0.6 n=30 agrees=18 more=2 less=10 unavail=0</t>
+          <t>value=0.6 n=10 agrees=6 more=1 less=2 unavail=1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -34241,7 +35223,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Patient fell suddenly and is unresponsive, indicating unconsciousness emergency</t>
+          <t>Sudden fall and unresponsive requires emergency ambulance.</t>
         </is>
       </c>
     </row>
@@ -34263,7 +35245,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>home_nursing</t>
+          <t>paramedic_home_visit</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -34273,7 +35255,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Request for injection at home; no red flags present</t>
+          <t>Patient needs an injection at home.</t>
         </is>
       </c>
     </row>
@@ -34293,21 +35275,12 @@
           <t>paramedic_home_visit</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>lab_test_home</t>
-        </is>
-      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>llm_less_severe_ignored</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Home monitoring of hypertension and diabetes requested, no acute red flags</t>
-        </is>
-      </c>
+          <t>llm_unavailable</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -34337,268 +35310,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Vague booking request; teleconsultation best first step to assess needs</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>S0016</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>papa ko tej sine men drd hai aur sans nhin aa rhi</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>paramedic_home_visit</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>emergency_112</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>llm_more_severe_asked</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Severe chest pain with breathlessness needs immediate emergency response</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>S0021</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>cbc aur thyroid test ghar se sample lekar</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>teleconsultation</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>lab_test_home</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>llm_less_severe_ignored</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Patient requests home sample collection for CBC and thyroid tests.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>S0023</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>subah se acidity gas hai doctor se consult karna hai</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>home_nursing</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>teleconsultation</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>llm_less_severe_ignored</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Acidity and gas since morning; suitable for doctor consultation, no red flags.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>S0025</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>my father has had fever and cough for 2 days</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>paramedic_home_visit</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>teleconsultation</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>llm_less_severe_ignored</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Fever and cough for 2 days, no red flags; teleconsultation appropriate</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>S0026</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>my father has had fever and cough for 2 days</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>paramedic_home_visit</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>teleconsultation</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>llm_less_severe_ignored</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Fever and cough for 2 days, no red flags; teleconsultation appropriate</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>S0029</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>kl subh shugr test ghr pr</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>teleconsultation</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>lab_test_home</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>llm_less_severe_ignored</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Patient requests home blood sugar test tomorrow morning</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>S0030</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>papa ko insulin lgvana hai</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>paramedic_home_visit</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>home_nursing</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>llm_less_severe_ignored</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Patient needs insulin injection administered at home by a nurse.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>S0037</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>ghr pr injekshn lgvana hai</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>teleconsultation</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>home_nursing</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>llm_less_severe_ignored</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Request for injection at home; no red flags present</t>
+          <t>No symptoms; teleconsultation for initial assessment.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F14"/>
+  <autoFilter ref="A1:F6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>